<commit_message>
feat: complete bank statement import feature
</commit_message>
<xml_diff>
--- a/昆山邦洁工业润滑油有限公司+进项+2025+04-06.xlsx
+++ b/昆山邦洁工业润滑油有限公司+进项+2025+04-06.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\公司文件\Office\Other\工业轮滑油\发票\邦洁发票\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI\ai-finance-assistant\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D79743-3A8E-492C-A57D-053737066005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7924D17B-BABE-44BD-BA51-4FC02EC1A0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="信息汇总表" sheetId="1" r:id="rId1"/>
@@ -354,7 +354,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -687,7 +687,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA8"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="11" width="22" customWidth="1"/>
@@ -700,7 +700,7 @@
     <col min="21" max="27" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="17.399999999999999" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -783,7 +783,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -864,7 +864,7 @@
       </c>
       <c r="AA2" s="2"/>
     </row>
-    <row r="3" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>47</v>
       </c>
@@ -941,7 +941,7 @@
       </c>
       <c r="AA3" s="2"/>
     </row>
-    <row r="4" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="AA4" s="2"/>
     </row>
-    <row r="5" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>65</v>
       </c>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="AA5" s="2"/>
     </row>
-    <row r="6" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>66</v>
       </c>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="AA6" s="2"/>
     </row>
-    <row r="7" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>39</v>
       </c>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="AA7" s="2"/>
     </row>
-    <row r="8" spans="1:27" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>73</v>
       </c>
@@ -1351,7 +1351,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:S7"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="9" width="22" customWidth="1"/>
@@ -1359,7 +1359,7 @@
     <col min="13" max="19" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="17.399999999999999" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="S2" s="2"/>
     </row>
-    <row r="3" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>47</v>
       </c>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="S3" s="2"/>
     </row>
-    <row r="4" spans="1:19" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="S4" s="2"/>
     </row>
-    <row r="5" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>65</v>
       </c>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="S5" s="2"/>
     </row>
-    <row r="6" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>66</v>
       </c>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="S6" s="2"/>
     </row>
-    <row r="7" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>77</v>
       </c>

</xml_diff>